<commit_message>
Update Verdigris model and deck with founder inputs
Product mix by funder (bridging £650k, development £1.25m at 30%),
analyst pay under £55k, and a salary benchmarks sheet showing industry
ranges beside the figures used. Deck figures re-synced to the model.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WiYieSwuhSHZ2QAH5RV2m7
</commit_message>
<xml_diff>
--- a/verdigris-deliverables/Verdigris_Economics_Model.xlsx
+++ b/verdigris-deliverables/Verdigris_Economics_Model.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Headcount - Traditional" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Headcount - AI-native" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Revenue" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Comparison" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Per-case cost" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headcount - Traditional" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headcount - AI-native" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary benchmarks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-case cost" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,10 +26,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="£#,##0;(£#,##0);-"/>
-    <numFmt numFmtId="165" formatCode="#,##0;(#,##0);-"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0;(#,##0.0);-"/>
-    <numFmt numFmtId="167" formatCode="0.00%;(0.00%);-"/>
-    <numFmt numFmtId="168" formatCode="0.0%;(0.0%);-"/>
+    <numFmt numFmtId="165" formatCode="0.0%;(0.0%);-"/>
+    <numFmt numFmtId="166" formatCode="#,##0;(#,##0);-"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0;(#,##0.0);-"/>
+    <numFmt numFmtId="168" formatCode="0.00%;(0.00%);-"/>
     <numFmt numFmtId="169" formatCode="0.0&quot;x&quot;"/>
   </numFmts>
   <fonts count="10">
@@ -150,28 +151,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -267,17 +268,17 @@
     </comment>
     <comment ref="E7" authorId="0" shapeId="0">
       <text>
-        <t>Senior bridging UW £70–80k + 10–20% (exec-appointments; Fintelligent).</t>
+        <t>Founder: analysts normally under £55k; seniors above. Market ads: senior bridging UW £65–80k (exec-appointments; Fintelligent). £65k used.</t>
       </text>
     </comment>
     <comment ref="E8" authorId="0" shapeId="0">
       <text>
-        <t>Mid UW £45–65k + 10–20% (Tandem; Fintelligent job ads).</t>
+        <t>Founder: credit analysts normally under £55k. Market ads: £45–65k + 10–20% (Tandem; Fintelligent). £50k used.</t>
       </text>
     </comment>
     <comment ref="E9" authorId="0" shapeId="0">
       <text>
-        <t>Junior bridging UW £30–45k (Fame Recruitment ad; talent.com).</t>
+        <t>Junior bridging UW £30–45k (Fame Recruitment ad; talent.com); founder: under £55k for analysts. £35k used.</t>
       </text>
     </comment>
     <comment ref="E10" authorId="0" shapeId="0">
@@ -688,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B27"/>
+  <dimension ref="B2:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -774,81 +775,95 @@
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>4. Revenue — revenue build for the loan book (identical for both models).</t>
+          <t>4. Salary benchmarks — industry ranges (low / mid / high) next to the figures used.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>5. Comparison — P&amp;L side by side, cost per loan, margin, and the scaling table (£150m → £600m book).</t>
+          <t>5. Revenue — revenue build for the loan book (identical for both models).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>6. Per-case cost — what it costs to underwrite ONE case, human vs AI-assisted.</t>
+          <t>6. Comparison — P&amp;L side by side, cost per loan, margin, and the scaling table (£150m → £600m book).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>7. Sources — where every number came from, with URLs.</t>
+          <t>7. Per-case cost — what it costs to underwrite ONE case, human vs AI-assisted.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>8. Sources — where every number came from, with URLs.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Status of the numbers</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>• Salary bands: 2025–26 London job ads and salary guides (see Sources). C-suite bands are estimates.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>• Loan book, loan size, completions: founder estimate calibrated to public market data (BDLA avg loan £540k; ~25 loans per analyst per year).</t>
+          <t>• Salary bands: 2025–26 London job ads and salary guides (see Sources). C-suite bands are estimates.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>• Pricing: market rates (0.81–0.84%/month average, Bridging Trends 2025–26). Arrangement fee and broker fee are market-typical assumptions.</t>
+          <t>• Loan sizes: founder — bridging/refurb £500–800k via institutional partner (≤£1m); ground-up development £1–1.5m via bank partner, a growing share. Book £150m is a founder estimate.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>• AI cost per case: computed from Anthropic list prices (June 2026) and typical document volumes; a 10x safety factor is applied.</t>
+          <t>• Analyst pay: founder — credit analysts normally under £55k; other roles from London 2025–26 benchmarks (Salary benchmarks sheet).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>• Nothing in this model is a claim about any specific company. 'Northgate Bridging' is a composite.</t>
+          <t>• Pricing: market rates (0.81–0.84%/month average, Bridging Trends 2025–26). Arrangement fee and broker fee are market-typical assumptions.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>• AI cost per case: computed from Anthropic list prices (June 2026) and typical document volumes; a 10x safety factor is applied.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>• Nothing in this model is a claim about any specific company. 'Northgate Bridging' is a composite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Built 9 September 2026.</t>
         </is>
@@ -865,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E41"/>
+  <dimension ref="B2:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -937,7 +952,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Average loan size</t>
+          <t>Bridging / refurbishment: average loan size</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
@@ -950,59 +965,58 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Founder data: pipeline tracker Jan 2026 shows facilities £205k–£1.59m, median ≈ £440k; development loans larger; CV: typically £500k–£1m. BDLA market average £540k.</t>
+          <t>Founder: funded by the institutional partner, normally up to £1m; typical property £500–800k. Pipeline tracker Jan 2026: facilities £205k–£1.59m, median ≈ £440k.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Average term</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>12</v>
+          <t>Ground-up development: average loan size</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1250000</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>months</t>
+          <t>£</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Bridging Trends 2025 average term 12 months; founder calculator example 18 months (refurb).</t>
+          <t>Founder: funded by the bank partner, typically £1m–£1.5m; a growing share of the book.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Loans completed per year</t>
-        </is>
-      </c>
-      <c r="C9" s="12">
-        <f>ROUND(C6/C7*12/C8,0)</f>
-        <v/>
+          <t>Share of originations that are ground-up development</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0.3</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>loans</t>
+          <t>% by count</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Book ÷ avg loan × 12 ÷ term. ~240 → ~24 per underwriter with 10 in credit, matching ~25 loans/yr per analyst.</t>
+          <t>Founder: 'getting more of those'; 30% assumed. Change to reflect the current mix.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Annual originations (£)</t>
-        </is>
-      </c>
-      <c r="C10" s="13">
-        <f>C9*C7</f>
+          <t>Blended average loan size</t>
+        </is>
+      </c>
+      <c r="C10" s="12">
+        <f>C7*(1-C9)+C8*C9</f>
         <v/>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -1012,190 +1026,192 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>Loans × average loan size.</t>
+          <t>Weighted by product mix.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Applications assessed per completed loan</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>4</v>
+          <t>Average term</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>12</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>months</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Founder estimate: pipeline of 15–23 live cases vs ~2 completions/month per analyst → roughly 1 in 4 assessed cases completes.</t>
+          <t>Bridging Trends 2025 average term 12 months; founder calculator example 18 months (refurb).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Cases assessed per year</t>
-        </is>
-      </c>
-      <c r="C12" s="12">
-        <f>C9*C11</f>
+          <t>Loans completed per year</t>
+        </is>
+      </c>
+      <c r="C12" s="14">
+        <f>ROUND(C6/C10*12/C11,0)</f>
         <v/>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>cases</t>
+          <t>loans</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>Every assessed case costs underwriting effort whether or not it completes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>PRICING &amp; REVENUE</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
+          <t>Book ÷ blended loan × 12 ÷ term. With 10 in credit ≈ 19 per underwriter, versus founder's ~25/yr as an analyst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Annual originations (£)</t>
+        </is>
+      </c>
+      <c r="C13" s="12">
+        <f>C12*C10</f>
+        <v/>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>£</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Loans × blended average loan size.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Borrower interest rate (monthly)</t>
+          <t>Applications assessed per completed loan</t>
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>0.008999999999999999</v>
+        <v>4</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>% / month</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator: 0.95%/month fixed on a medium refurb (variable option BoE 4.25% + 0.51%/mo = 10.37% pa). Market average 0.81–0.84% (Bridging Trends). 0.90% blended used.</t>
+          <t>Founder estimate: pipeline of 15–23 live cases vs ~2 completions/month per analyst → roughly 1 in 4 assessed cases completes.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Borrower interest rate (annualised, simple)</t>
-        </is>
-      </c>
-      <c r="C15" s="16">
-        <f>C14*12</f>
+          <t>Cases assessed per year</t>
+        </is>
+      </c>
+      <c r="C15" s="14">
+        <f>C12*C14</f>
         <v/>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>% pa</t>
+          <t>cases</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Simple ×12. Founder calculator effective rate 11.98% pa on 0.95%/mo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Arrangement fee charged to borrower</t>
-        </is>
-      </c>
-      <c r="C16" s="17" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>% of loan</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Founder calculator: 2% of gross loan ('Lender &amp; Broker Fee').</t>
-        </is>
-      </c>
+          <t>Every assessed case costs underwriting effort whether or not it completes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>PRICING &amp; REVENUE</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Arrangement fee retained by lender (after introducer share)</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="n">
-        <v>0.005</v>
+          <t>Borrower interest rate (monthly)</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>0.008999999999999999</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>% of loan</t>
+          <t>% / month</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator: on the example deal 0% retained, 2% paid as 'introducer share'. Founder: broker payout 1–2%. 0.5% retained assumed — change if your typical split differs.</t>
+          <t>Founder calculator: 0.95%/month fixed on a medium refurb (variable option BoE 4.25% + 0.51%/mo = 10.37% pa). Market average 0.81–0.84% (Bridging Trends). 0.90% blended used.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Admin fee per loan (retained)</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="n">
-        <v>1500</v>
+          <t>Borrower interest rate (annualised, simple)</t>
+        </is>
+      </c>
+      <c r="C18" s="17">
+        <f>C17*12</f>
+        <v/>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>£</t>
+          <t>% pa</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator: £1,995 (&lt;£100k), £1,500 (£100–250k), £1,250 (&gt;£250k) automatic admin fee. £1,500 blended.</t>
+          <t>Simple ×12. Founder calculator effective rate 11.98% pa on 0.95%/mo.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Redemption + drawdown fees per loan</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="n">
-        <v>1500</v>
+          <t>Arrangement fee charged to borrower</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>0.02</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>£</t>
+          <t>% of loan</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator: redemption fee £495; drawdown fee £295/month on refurb/development. ~£1,500 per loan blended.</t>
+          <t>Founder calculator: 2% of gross loan ('Lender &amp; Broker Fee').</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Exit fee</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="n">
-        <v>0</v>
+          <t>Arrangement fee retained by lender (after introducer share)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>0.005</v>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
@@ -1204,88 +1220,98 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator: 0%. Some lenders charge 0–1%.</t>
+          <t>Founder calculator: on the example deal 0% retained, 2% paid as 'introducer share'. Founder: broker payout 1–2%. 0.5% retained assumed — change if your typical split differs.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Other fees (extension, variation, non-redemption)</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="n">
-        <v>0.002</v>
+          <t>Admin fee per loan (retained)</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>1500</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>% of originations</t>
+          <t>£</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Founder estimate; extension/variation fees exist but are not systematic.</t>
+          <t>Founder calculator: £1,995 (&lt;£100k), £1,500 (£100–250k), £1,250 (&gt;£250k) automatic admin fee. £1,500 blended.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Share of loans introduced by brokers</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="n">
-        <v>0.85</v>
+          <t>Redemption + drawdown fees per loan</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="n">
+        <v>1500</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>BDLA/Interpath 2026 survey: 61% of lenders name brokers as primary channel, 15% direct → ~85% broker-introduced. Broker fee is already netted in 'retained' above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>FUNDING &amp; RISK</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
+          <t>Founder calculator: redemption fee £495; drawdown fee £295/month on refurb/development. ~£1,500 per loan blended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Exit fee</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>% of loan</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Founder calculator: 0%. Some lenders charge 0–1%.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Funding partner buy rate (cost of funds, annual)</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="n">
-        <v>0.08749999999999999</v>
+          <t>Other fees (extension, variation, non-redemption)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>0.002</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>% pa</t>
+          <t>% of originations</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator rate card: institutional partner 8.25–9.75% depending on product and advance rate (8.75% on the example); bank line = BoE + 4.3–4.8%. 8.75% used.</t>
+          <t>Founder estimate; extension/variation fees exist but are not systematic.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Share of book funded by partners</t>
+          <t>Share of loans introduced by brokers</t>
         </is>
       </c>
       <c r="C25" s="19" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
@@ -1294,38 +1320,28 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Founder calculator: partner advance rate 95%, lender first-loss 5%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Funder fee per loan</t>
-        </is>
-      </c>
-      <c r="C26" s="18" t="n">
-        <v>500</v>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>£</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>Founder calculator: £500 partner fee per deal.</t>
-        </is>
-      </c>
+          <t>BDLA/Interpath 2026 survey: 61% of lenders name brokers as primary channel, 15% direct → ~85% broker-introduced. Broker fee is already netted in 'retained' above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>FUNDING &amp; RISK</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Expected credit loss (annual, % of book)</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="n">
-        <v>0.005</v>
+          <t>Funding partner buy rate (cost of funds, annual)</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>0.08749999999999999</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -1334,108 +1350,108 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Founder estimate; comparator claims 0 capital losses over 7 years; BDLA default rates typically &lt;1%. 0.5% is prudent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>EMPLOYMENT ON-COSTS (2026/27)</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
+          <t>Founder calculator rate card: institutional partner 8.25–9.75% depending on product and advance rate (8.75% on the example); bank line = BoE + 4.3–4.8%. 8.75% used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Share of book funded by partners</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Founder calculator: partner advance rate 95%, lender first-loss 5%.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Employer National Insurance rate</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="n">
-        <v>0.15</v>
+          <t>Funder fee per loan</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="n">
+        <v>500</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>15% above secondary threshold (unchanged from April 2025).</t>
+          <t>Founder calculator: £500 partner fee per deal.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>NI secondary threshold</t>
-        </is>
-      </c>
-      <c r="C30" s="18" t="n">
-        <v>5000</v>
+          <t>Expected credit loss (annual, % of book)</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="n">
+        <v>0.005</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>£ pa</t>
+          <t>% pa</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>£5,000 per employee per year, frozen to 2030–31.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Employer pension contribution</t>
-        </is>
-      </c>
-      <c r="C31" s="19" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>% of salary</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Auto-enrolment minimum 3%; 5% typical for a financial-services employer.</t>
-        </is>
-      </c>
+          <t>Founder estimate; comparator claims 0 capital losses over 7 years; BDLA default rates typically &lt;1%. 0.5% is prudent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>EMPLOYMENT ON-COSTS (2026/27)</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Other on-costs (benefits, kit, recruitment, software seats)</t>
+          <t>Employer National Insurance rate</t>
         </is>
       </c>
       <c r="C32" s="19" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>% of salary</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>All-in multiplier 1.25–1.4x is typical (Grove HR); NI 15% + pension 5% + 8% other ≈ 1.28x.</t>
+          <t>15% above secondary threshold (unchanged from April 2025).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Office cost per desk per year</t>
+          <t>NI secondary threshold</t>
         </is>
       </c>
       <c r="C33" s="18" t="n">
-        <v>9600</v>
+        <v>5000</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -1444,155 +1460,215 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>London serviced office £700–900/desk/month City; £800 used.</t>
+          <t>£5,000 per employee per year, frozen to 2030–31.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Software &amp; data per employee per year</t>
-        </is>
-      </c>
-      <c r="C34" s="18" t="n">
-        <v>3000</v>
+          <t>Employer pension contribution</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>0.05</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>£ pa</t>
+          <t>% of salary</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>CRM/LOS seat £1–3k plus general tooling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>AI-NATIVE OPERATING COSTS</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
+          <t>Auto-enrolment minimum 3%; 5% typical for a financial-services employer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Other on-costs (benefits, kit, recruitment, software seats)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>% of salary</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>All-in multiplier 1.25–1.4x is typical (Grove HR); NI 15% + pension 5% + 8% other ≈ 1.28x.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Model (LLM) cost per assessed case</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n">
-        <v>16</v>
+          <t>Office cost per desk per year</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="n">
+        <v>9600</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>£</t>
+          <t>£ pa</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>Anthropic list prices Jun 2026: Opus 5 $5/$25 per M tokens; ~300k input + 20k output tokens per case ≈ $2. ×10 safety factor for retries, tools, re-underwrites, evals = $20 ≈ £16 at $1.30/£.</t>
+          <t>London serviced office £700–900/desk/month City; £800 used.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Data &amp; verification per assessed case</t>
+          <t>Software &amp; data per employee per year</t>
         </is>
       </c>
       <c r="C37" s="18" t="n">
-        <v>50</v>
+        <v>3000</v>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>£</t>
+          <t>£ pa</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>Land Registry £7/doc (£14–28), KYC £2–6, company credit £5–15, AVM £10–25, consumer credit £1–5 → £40–80.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Platform, hosting, monitoring per year</t>
-        </is>
-      </c>
-      <c r="C38" s="18" t="n">
-        <v>60000</v>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>£ pa</t>
-        </is>
-      </c>
-      <c r="E38" s="10" t="inlineStr">
-        <is>
-          <t>Founder estimate: cloud, observability, model evals, security tooling for a regulated lender.</t>
-        </is>
-      </c>
+          <t>CRM/LOS seat £1–3k plus general tooling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>AI-NATIVE OPERATING COSTS</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Human review time per assessed case (AI-native)</t>
-        </is>
-      </c>
-      <c r="C39" s="14" t="n">
-        <v>1.5</v>
+          <t>Model (LLM) cost per assessed case</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="n">
+        <v>16</v>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>£</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Underwriter reviews the AI-drafted pack and decides. Founder estimate.</t>
+          <t>Anthropic list prices Jun 2026: Opus 5 $5/$25 per M tokens; ~300k input + 20k output tokens per case ≈ $2. ×10 safety factor for retries, tools, re-underwrites, evals = $20 ≈ £16 at $1.30/£.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Underwriter time per assessed case (traditional)</t>
-        </is>
-      </c>
-      <c r="C40" s="20" t="n">
-        <v>12</v>
+          <t>Data &amp; verification per assessed case</t>
+        </is>
+      </c>
+      <c r="C40" s="18" t="n">
+        <v>50</v>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>£</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>Founder estimate: 15–23 live cases, ~2 completions/month, ~50% of week on document work. Includes reading, reconciling, chasing, credit paper.</t>
+          <t>Land Registry £7/doc (£14–28), KYC £2–6, company credit £5–15, AVM £10–25, consumer credit £1–5 → £40–80.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="B41" s="7" t="inlineStr">
         <is>
+          <t>Platform, hosting, monitoring per year</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>£ pa</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Founder estimate: cloud, observability, model evals, security tooling for a regulated lender.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Human review time per assessed case (AI-native)</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>Underwriter reviews the AI-drafted pack and decides. Founder estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Underwriter time per assessed case (traditional)</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Founder estimate: 15–23 live cases, ~2 completions/month, ~50% of week on document work. Includes reading, reconciling, chasing, credit paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
           <t>Working hours per FTE per year</t>
         </is>
       </c>
-      <c r="C41" s="11" t="n">
+      <c r="C44" s="13" t="n">
         <v>1650</v>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D44" s="9" t="inlineStr">
         <is>
           <t>hours</t>
         </is>
       </c>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="E44" s="10" t="inlineStr">
         <is>
           <t>37.5 h/week × 44 productive weeks.</t>
         </is>
@@ -1708,7 +1784,7 @@
           <t>Head of Credit</t>
         </is>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="18" t="n">
@@ -1717,23 +1793,23 @@
       <c r="F6" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="12">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="12">
         <f>G6*F6</f>
         <v/>
       </c>
-      <c r="I6" s="13">
-        <f>MAX(0,(E6+E6*F6)-Assumptions!$C$30)*Assumptions!$C$29*D6</f>
-        <v/>
-      </c>
-      <c r="J6" s="13">
-        <f>(G6+H6)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K6" s="13">
+      <c r="I6" s="12">
+        <f>MAX(0,(E6+E6*F6)-Assumptions!$C$33)*Assumptions!$C$32*D6</f>
+        <v/>
+      </c>
+      <c r="J6" s="12">
+        <f>(G6+H6)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K6" s="12">
         <f>G6+H6+I6+J6</f>
         <v/>
       </c>
@@ -1754,38 +1830,38 @@
           <t>Senior underwriter (bridging + development)</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>75000</v>
+        <v>65000</v>
       </c>
       <c r="F7" s="19" t="n">
         <v>0.15</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="12">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="12">
         <f>G7*F7</f>
         <v/>
       </c>
-      <c r="I7" s="13">
-        <f>MAX(0,(E7+E7*F7)-Assumptions!$C$30)*Assumptions!$C$29*D7</f>
-        <v/>
-      </c>
-      <c r="J7" s="13">
-        <f>(G7+H7)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K7" s="13">
+      <c r="I7" s="12">
+        <f>MAX(0,(E7+E7*F7)-Assumptions!$C$33)*Assumptions!$C$32*D7</f>
+        <v/>
+      </c>
+      <c r="J7" s="12">
+        <f>(G7+H7)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K7" s="12">
         <f>G7+H7+I7+J7</f>
         <v/>
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>Senior bridging UW £70–80k + 10–20% (exec-appointments; Fintelligent).</t>
+          <t>Founder: analysts normally under £55k; seniors above. Market ads: senior bridging UW £65–80k (exec-appointments; Fintelligent). £65k used.</t>
         </is>
       </c>
     </row>
@@ -1800,38 +1876,38 @@
           <t>Credit analyst / underwriter (mid)</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>4</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>55000</v>
+        <v>50000</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G8" s="13">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="12">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="12">
         <f>G8*F8</f>
         <v/>
       </c>
-      <c r="I8" s="13">
-        <f>MAX(0,(E8+E8*F8)-Assumptions!$C$30)*Assumptions!$C$29*D8</f>
-        <v/>
-      </c>
-      <c r="J8" s="13">
-        <f>(G8+H8)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K8" s="13">
+      <c r="I8" s="12">
+        <f>MAX(0,(E8+E8*F8)-Assumptions!$C$33)*Assumptions!$C$32*D8</f>
+        <v/>
+      </c>
+      <c r="J8" s="12">
+        <f>(G8+H8)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K8" s="12">
         <f>G8+H8+I8+J8</f>
         <v/>
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Mid UW £45–65k + 10–20% (Tandem; Fintelligent job ads).</t>
+          <t>Founder: credit analysts normally under £55k. Market ads: £45–65k + 10–20% (Tandem; Fintelligent). £50k used.</t>
         </is>
       </c>
     </row>
@@ -1846,38 +1922,38 @@
           <t>Junior credit analyst</t>
         </is>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>3</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>37500</v>
+        <v>35000</v>
       </c>
       <c r="F9" s="19" t="n">
         <v>0.05</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="12">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="12">
         <f>G9*F9</f>
         <v/>
       </c>
-      <c r="I9" s="13">
-        <f>MAX(0,(E9+E9*F9)-Assumptions!$C$30)*Assumptions!$C$29*D9</f>
-        <v/>
-      </c>
-      <c r="J9" s="13">
-        <f>(G9+H9)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K9" s="13">
+      <c r="I9" s="12">
+        <f>MAX(0,(E9+E9*F9)-Assumptions!$C$33)*Assumptions!$C$32*D9</f>
+        <v/>
+      </c>
+      <c r="J9" s="12">
+        <f>(G9+H9)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K9" s="12">
         <f>G9+H9+I9+J9</f>
         <v/>
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>Junior bridging UW £30–45k (Fame Recruitment ad; talent.com).</t>
+          <t>Junior bridging UW £30–45k (Fame Recruitment ad; talent.com); founder: under £55k for analysts. £35k used.</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1968,7 @@
           <t>Portfolio manager</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="18" t="n">
@@ -1901,23 +1977,23 @@
       <c r="F10" s="19" t="n">
         <v>0.125</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="12">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="12">
         <f>G10*F10</f>
         <v/>
       </c>
-      <c r="I10" s="13">
-        <f>MAX(0,(E10+E10*F10)-Assumptions!$C$30)*Assumptions!$C$29*D10</f>
-        <v/>
-      </c>
-      <c r="J10" s="13">
-        <f>(G10+H10)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K10" s="13">
+      <c r="I10" s="12">
+        <f>MAX(0,(E10+E10*F10)-Assumptions!$C$33)*Assumptions!$C$32*D10</f>
+        <v/>
+      </c>
+      <c r="J10" s="12">
+        <f>(G10+H10)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K10" s="12">
         <f>G10+H10+I10+J10</f>
         <v/>
       </c>
@@ -1938,7 +2014,7 @@
           <t>Completions / case manager</t>
         </is>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>3</v>
       </c>
       <c r="E11" s="18" t="n">
@@ -1947,23 +2023,23 @@
       <c r="F11" s="19" t="n">
         <v>0.05</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="12">
         <f>D11*E11</f>
         <v/>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="12">
         <f>G11*F11</f>
         <v/>
       </c>
-      <c r="I11" s="13">
-        <f>MAX(0,(E11+E11*F11)-Assumptions!$C$30)*Assumptions!$C$29*D11</f>
-        <v/>
-      </c>
-      <c r="J11" s="13">
-        <f>(G11+H11)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K11" s="13">
+      <c r="I11" s="12">
+        <f>MAX(0,(E11+E11*F11)-Assumptions!$C$33)*Assumptions!$C$32*D11</f>
+        <v/>
+      </c>
+      <c r="J11" s="12">
+        <f>(G11+H11)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K11" s="12">
         <f>G11+H11+I11+J11</f>
         <v/>
       </c>
@@ -1984,7 +2060,7 @@
           <t>Loan administrator / servicing</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>4</v>
       </c>
       <c r="E12" s="18" t="n">
@@ -1993,23 +2069,23 @@
       <c r="F12" s="19" t="n">
         <v>0.025</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="12">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="12">
         <f>G12*F12</f>
         <v/>
       </c>
-      <c r="I12" s="13">
-        <f>MAX(0,(E12+E12*F12)-Assumptions!$C$30)*Assumptions!$C$29*D12</f>
-        <v/>
-      </c>
-      <c r="J12" s="13">
-        <f>(G12+H12)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K12" s="13">
+      <c r="I12" s="12">
+        <f>MAX(0,(E12+E12*F12)-Assumptions!$C$33)*Assumptions!$C$32*D12</f>
+        <v/>
+      </c>
+      <c r="J12" s="12">
+        <f>(G12+H12)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K12" s="12">
         <f>G12+H12+I12+J12</f>
         <v/>
       </c>
@@ -2030,7 +2106,7 @@
           <t>Head of Sales</t>
         </is>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="n">
@@ -2039,23 +2115,23 @@
       <c r="F13" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="12">
         <f>D13*E13</f>
         <v/>
       </c>
-      <c r="H13" s="13">
+      <c r="H13" s="12">
         <f>G13*F13</f>
         <v/>
       </c>
-      <c r="I13" s="13">
-        <f>MAX(0,(E13+E13*F13)-Assumptions!$C$30)*Assumptions!$C$29*D13</f>
-        <v/>
-      </c>
-      <c r="J13" s="13">
-        <f>(G13+H13)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K13" s="13">
+      <c r="I13" s="12">
+        <f>MAX(0,(E13+E13*F13)-Assumptions!$C$33)*Assumptions!$C$32*D13</f>
+        <v/>
+      </c>
+      <c r="J13" s="12">
+        <f>(G13+H13)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K13" s="12">
         <f>G13+H13+I13+J13</f>
         <v/>
       </c>
@@ -2076,7 +2152,7 @@
           <t>Senior BDM / originator</t>
         </is>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E14" s="18" t="n">
@@ -2085,23 +2161,23 @@
       <c r="F14" s="19" t="n">
         <v>0.6</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="12">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="H14" s="13">
+      <c r="H14" s="12">
         <f>G14*F14</f>
         <v/>
       </c>
-      <c r="I14" s="13">
-        <f>MAX(0,(E14+E14*F14)-Assumptions!$C$30)*Assumptions!$C$29*D14</f>
-        <v/>
-      </c>
-      <c r="J14" s="13">
-        <f>(G14+H14)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K14" s="13">
+      <c r="I14" s="12">
+        <f>MAX(0,(E14+E14*F14)-Assumptions!$C$33)*Assumptions!$C$32*D14</f>
+        <v/>
+      </c>
+      <c r="J14" s="12">
+        <f>(G14+H14)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K14" s="12">
         <f>G14+H14+I14+J14</f>
         <v/>
       </c>
@@ -2122,7 +2198,7 @@
           <t>BDM</t>
         </is>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="15" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="18" t="n">
@@ -2131,23 +2207,23 @@
       <c r="F15" s="19" t="n">
         <v>0.4</v>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="12">
         <f>D15*E15</f>
         <v/>
       </c>
-      <c r="H15" s="13">
+      <c r="H15" s="12">
         <f>G15*F15</f>
         <v/>
       </c>
-      <c r="I15" s="13">
-        <f>MAX(0,(E15+E15*F15)-Assumptions!$C$30)*Assumptions!$C$29*D15</f>
-        <v/>
-      </c>
-      <c r="J15" s="13">
-        <f>(G15+H15)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K15" s="13">
+      <c r="I15" s="12">
+        <f>MAX(0,(E15+E15*F15)-Assumptions!$C$33)*Assumptions!$C$32*D15</f>
+        <v/>
+      </c>
+      <c r="J15" s="12">
+        <f>(G15+H15)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K15" s="12">
         <f>G15+H15+I15+J15</f>
         <v/>
       </c>
@@ -2168,7 +2244,7 @@
           <t>Marketing manager</t>
         </is>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="18" t="n">
@@ -2177,23 +2253,23 @@
       <c r="F16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="12">
         <f>D16*E16</f>
         <v/>
       </c>
-      <c r="H16" s="13">
+      <c r="H16" s="12">
         <f>G16*F16</f>
         <v/>
       </c>
-      <c r="I16" s="13">
-        <f>MAX(0,(E16+E16*F16)-Assumptions!$C$30)*Assumptions!$C$29*D16</f>
-        <v/>
-      </c>
-      <c r="J16" s="13">
-        <f>(G16+H16)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K16" s="13">
+      <c r="I16" s="12">
+        <f>MAX(0,(E16+E16*F16)-Assumptions!$C$33)*Assumptions!$C$32*D16</f>
+        <v/>
+      </c>
+      <c r="J16" s="12">
+        <f>(G16+H16)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K16" s="12">
         <f>G16+H16+I16+J16</f>
         <v/>
       </c>
@@ -2214,7 +2290,7 @@
           <t>Marketing executive</t>
         </is>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="15" t="n">
         <v>3</v>
       </c>
       <c r="E17" s="18" t="n">
@@ -2223,23 +2299,23 @@
       <c r="F17" s="19" t="n">
         <v>0.025</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17" s="12">
         <f>D17*E17</f>
         <v/>
       </c>
-      <c r="H17" s="13">
+      <c r="H17" s="12">
         <f>G17*F17</f>
         <v/>
       </c>
-      <c r="I17" s="13">
-        <f>MAX(0,(E17+E17*F17)-Assumptions!$C$30)*Assumptions!$C$29*D17</f>
-        <v/>
-      </c>
-      <c r="J17" s="13">
-        <f>(G17+H17)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K17" s="13">
+      <c r="I17" s="12">
+        <f>MAX(0,(E17+E17*F17)-Assumptions!$C$33)*Assumptions!$C$32*D17</f>
+        <v/>
+      </c>
+      <c r="J17" s="12">
+        <f>(G17+H17)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K17" s="12">
         <f>G17+H17+I17+J17</f>
         <v/>
       </c>
@@ -2260,7 +2336,7 @@
           <t>CEO / Managing Director</t>
         </is>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="18" t="n">
@@ -2269,23 +2345,23 @@
       <c r="F18" s="19" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18" s="12">
         <f>D18*E18</f>
         <v/>
       </c>
-      <c r="H18" s="13">
+      <c r="H18" s="12">
         <f>G18*F18</f>
         <v/>
       </c>
-      <c r="I18" s="13">
-        <f>MAX(0,(E18+E18*F18)-Assumptions!$C$30)*Assumptions!$C$29*D18</f>
-        <v/>
-      </c>
-      <c r="J18" s="13">
-        <f>(G18+H18)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K18" s="13">
+      <c r="I18" s="12">
+        <f>MAX(0,(E18+E18*F18)-Assumptions!$C$33)*Assumptions!$C$32*D18</f>
+        <v/>
+      </c>
+      <c r="J18" s="12">
+        <f>(G18+H18)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K18" s="12">
         <f>G18+H18+I18+J18</f>
         <v/>
       </c>
@@ -2306,7 +2382,7 @@
           <t>CFO / Finance Director</t>
         </is>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="18" t="n">
@@ -2315,23 +2391,23 @@
       <c r="F19" s="19" t="n">
         <v>0.225</v>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="12">
         <f>D19*E19</f>
         <v/>
       </c>
-      <c r="H19" s="13">
+      <c r="H19" s="12">
         <f>G19*F19</f>
         <v/>
       </c>
-      <c r="I19" s="13">
-        <f>MAX(0,(E19+E19*F19)-Assumptions!$C$30)*Assumptions!$C$29*D19</f>
-        <v/>
-      </c>
-      <c r="J19" s="13">
-        <f>(G19+H19)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K19" s="13">
+      <c r="I19" s="12">
+        <f>MAX(0,(E19+E19*F19)-Assumptions!$C$33)*Assumptions!$C$32*D19</f>
+        <v/>
+      </c>
+      <c r="J19" s="12">
+        <f>(G19+H19)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K19" s="12">
         <f>G19+H19+I19+J19</f>
         <v/>
       </c>
@@ -2352,7 +2428,7 @@
           <t>COO / Operations Director</t>
         </is>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="18" t="n">
@@ -2361,23 +2437,23 @@
       <c r="F20" s="19" t="n">
         <v>0.225</v>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="12">
         <f>D20*E20</f>
         <v/>
       </c>
-      <c r="H20" s="13">
+      <c r="H20" s="12">
         <f>G20*F20</f>
         <v/>
       </c>
-      <c r="I20" s="13">
-        <f>MAX(0,(E20+E20*F20)-Assumptions!$C$30)*Assumptions!$C$29*D20</f>
-        <v/>
-      </c>
-      <c r="J20" s="13">
-        <f>(G20+H20)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K20" s="13">
+      <c r="I20" s="12">
+        <f>MAX(0,(E20+E20*F20)-Assumptions!$C$33)*Assumptions!$C$32*D20</f>
+        <v/>
+      </c>
+      <c r="J20" s="12">
+        <f>(G20+H20)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K20" s="12">
         <f>G20+H20+I20+J20</f>
         <v/>
       </c>
@@ -2398,7 +2474,7 @@
           <t>CTO / Head of Technology</t>
         </is>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="D21" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="18" t="n">
@@ -2407,23 +2483,23 @@
       <c r="F21" s="19" t="n">
         <v>0.15</v>
       </c>
-      <c r="G21" s="13">
+      <c r="G21" s="12">
         <f>D21*E21</f>
         <v/>
       </c>
-      <c r="H21" s="13">
+      <c r="H21" s="12">
         <f>G21*F21</f>
         <v/>
       </c>
-      <c r="I21" s="13">
-        <f>MAX(0,(E21+E21*F21)-Assumptions!$C$30)*Assumptions!$C$29*D21</f>
-        <v/>
-      </c>
-      <c r="J21" s="13">
-        <f>(G21+H21)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K21" s="13">
+      <c r="I21" s="12">
+        <f>MAX(0,(E21+E21*F21)-Assumptions!$C$33)*Assumptions!$C$32*D21</f>
+        <v/>
+      </c>
+      <c r="J21" s="12">
+        <f>(G21+H21)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K21" s="12">
         <f>G21+H21+I21+J21</f>
         <v/>
       </c>
@@ -2444,7 +2520,7 @@
           <t>Compliance officer (SMF16/17)</t>
         </is>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="D22" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="18" t="n">
@@ -2453,23 +2529,23 @@
       <c r="F22" s="19" t="n">
         <v>0.125</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="12">
         <f>D22*E22</f>
         <v/>
       </c>
-      <c r="H22" s="13">
+      <c r="H22" s="12">
         <f>G22*F22</f>
         <v/>
       </c>
-      <c r="I22" s="13">
-        <f>MAX(0,(E22+E22*F22)-Assumptions!$C$30)*Assumptions!$C$29*D22</f>
-        <v/>
-      </c>
-      <c r="J22" s="13">
-        <f>(G22+H22)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K22" s="13">
+      <c r="I22" s="12">
+        <f>MAX(0,(E22+E22*F22)-Assumptions!$C$33)*Assumptions!$C$32*D22</f>
+        <v/>
+      </c>
+      <c r="J22" s="12">
+        <f>(G22+H22)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K22" s="12">
         <f>G22+H22+I22+J22</f>
         <v/>
       </c>
@@ -2490,7 +2566,7 @@
           <t>Software engineer / IT</t>
         </is>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="D23" s="15" t="n">
         <v>4</v>
       </c>
       <c r="E23" s="18" t="n">
@@ -2499,23 +2575,23 @@
       <c r="F23" s="19" t="n">
         <v>0.05</v>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="12">
         <f>D23*E23</f>
         <v/>
       </c>
-      <c r="H23" s="13">
+      <c r="H23" s="12">
         <f>G23*F23</f>
         <v/>
       </c>
-      <c r="I23" s="13">
-        <f>MAX(0,(E23+E23*F23)-Assumptions!$C$30)*Assumptions!$C$29*D23</f>
-        <v/>
-      </c>
-      <c r="J23" s="13">
-        <f>(G23+H23)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K23" s="13">
+      <c r="I23" s="12">
+        <f>MAX(0,(E23+E23*F23)-Assumptions!$C$33)*Assumptions!$C$32*D23</f>
+        <v/>
+      </c>
+      <c r="J23" s="12">
+        <f>(G23+H23)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K23" s="12">
         <f>G23+H23+I23+J23</f>
         <v/>
       </c>
@@ -2563,7 +2639,7 @@
         </is>
       </c>
       <c r="K26" s="24">
-        <f>D24*Assumptions!$C$33</f>
+        <f>D24*Assumptions!$C$36</f>
         <v/>
       </c>
     </row>
@@ -2574,7 +2650,7 @@
         </is>
       </c>
       <c r="K27" s="24">
-        <f>D24*Assumptions!$C$34</f>
+        <f>D24*Assumptions!$C$37</f>
         <v/>
       </c>
     </row>
@@ -2585,7 +2661,7 @@
         </is>
       </c>
       <c r="K28" s="24">
-        <f>Assumptions!$C$12*Assumptions!$C$37</f>
+        <f>Assumptions!$C$15*Assumptions!$C$40</f>
         <v/>
       </c>
     </row>
@@ -2700,7 +2776,7 @@
           <t>CEO / Head of Credit (founder, underwrites)</t>
         </is>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="18" t="n">
@@ -2709,23 +2785,23 @@
       <c r="F6" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="12">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="12">
         <f>G6*F6</f>
         <v/>
       </c>
-      <c r="I6" s="13">
-        <f>MAX(0,(E6+E6*F6)-Assumptions!$C$30)*Assumptions!$C$29*D6</f>
-        <v/>
-      </c>
-      <c r="J6" s="13">
-        <f>(G6+H6)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K6" s="13">
+      <c r="I6" s="12">
+        <f>MAX(0,(E6+E6*F6)-Assumptions!$C$33)*Assumptions!$C$32*D6</f>
+        <v/>
+      </c>
+      <c r="J6" s="12">
+        <f>(G6+H6)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K6" s="12">
         <f>G6+H6+I6+J6</f>
         <v/>
       </c>
@@ -2746,7 +2822,7 @@
           <t>CTO (technical co-founder)</t>
         </is>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="18" t="n">
@@ -2755,23 +2831,23 @@
       <c r="F7" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="12">
         <f>D7*E7</f>
         <v/>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="12">
         <f>G7*F7</f>
         <v/>
       </c>
-      <c r="I7" s="13">
-        <f>MAX(0,(E7+E7*F7)-Assumptions!$C$30)*Assumptions!$C$29*D7</f>
-        <v/>
-      </c>
-      <c r="J7" s="13">
-        <f>(G7+H7)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K7" s="13">
+      <c r="I7" s="12">
+        <f>MAX(0,(E7+E7*F7)-Assumptions!$C$33)*Assumptions!$C$32*D7</f>
+        <v/>
+      </c>
+      <c r="J7" s="12">
+        <f>(G7+H7)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K7" s="12">
         <f>G7+H7+I7+J7</f>
         <v/>
       </c>
@@ -2792,32 +2868,32 @@
           <t>Senior underwriter (human-in-the-loop)</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>75000</v>
+        <v>65000</v>
       </c>
       <c r="F8" s="19" t="n">
         <v>0.15</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="12">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="12">
         <f>G8*F8</f>
         <v/>
       </c>
-      <c r="I8" s="13">
-        <f>MAX(0,(E8+E8*F8)-Assumptions!$C$30)*Assumptions!$C$29*D8</f>
-        <v/>
-      </c>
-      <c r="J8" s="13">
-        <f>(G8+H8)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K8" s="13">
+      <c r="I8" s="12">
+        <f>MAX(0,(E8+E8*F8)-Assumptions!$C$33)*Assumptions!$C$32*D8</f>
+        <v/>
+      </c>
+      <c r="J8" s="12">
+        <f>(G8+H8)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K8" s="12">
         <f>G8+H8+I8+J8</f>
         <v/>
       </c>
@@ -2838,7 +2914,7 @@
           <t>Completions &amp; servicing lead</t>
         </is>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="18" t="n">
@@ -2847,23 +2923,23 @@
       <c r="F9" s="19" t="n">
         <v>0.05</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="12">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="12">
         <f>G9*F9</f>
         <v/>
       </c>
-      <c r="I9" s="13">
-        <f>MAX(0,(E9+E9*F9)-Assumptions!$C$30)*Assumptions!$C$29*D9</f>
-        <v/>
-      </c>
-      <c r="J9" s="13">
-        <f>(G9+H9)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K9" s="13">
+      <c r="I9" s="12">
+        <f>MAX(0,(E9+E9*F9)-Assumptions!$C$33)*Assumptions!$C$32*D9</f>
+        <v/>
+      </c>
+      <c r="J9" s="12">
+        <f>(G9+H9)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K9" s="12">
         <f>G9+H9+I9+J9</f>
         <v/>
       </c>
@@ -2884,7 +2960,7 @@
           <t>Compliance officer (SMF16/17)</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="18" t="n">
@@ -2893,23 +2969,23 @@
       <c r="F10" s="19" t="n">
         <v>0.125</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="12">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="12">
         <f>G10*F10</f>
         <v/>
       </c>
-      <c r="I10" s="13">
-        <f>MAX(0,(E10+E10*F10)-Assumptions!$C$30)*Assumptions!$C$29*D10</f>
-        <v/>
-      </c>
-      <c r="J10" s="13">
-        <f>(G10+H10)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K10" s="13">
+      <c r="I10" s="12">
+        <f>MAX(0,(E10+E10*F10)-Assumptions!$C$33)*Assumptions!$C$32*D10</f>
+        <v/>
+      </c>
+      <c r="J10" s="12">
+        <f>(G10+H10)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K10" s="12">
         <f>G10+H10+I10+J10</f>
         <v/>
       </c>
@@ -2930,7 +3006,7 @@
           <t>BDM / broker relationships</t>
         </is>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="18" t="n">
@@ -2939,23 +3015,23 @@
       <c r="F11" s="19" t="n">
         <v>0.4</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="12">
         <f>D11*E11</f>
         <v/>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="12">
         <f>G11*F11</f>
         <v/>
       </c>
-      <c r="I11" s="13">
-        <f>MAX(0,(E11+E11*F11)-Assumptions!$C$30)*Assumptions!$C$29*D11</f>
-        <v/>
-      </c>
-      <c r="J11" s="13">
-        <f>(G11+H11)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K11" s="13">
+      <c r="I11" s="12">
+        <f>MAX(0,(E11+E11*F11)-Assumptions!$C$33)*Assumptions!$C$32*D11</f>
+        <v/>
+      </c>
+      <c r="J11" s="12">
+        <f>(G11+H11)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K11" s="12">
         <f>G11+H11+I11+J11</f>
         <v/>
       </c>
@@ -2976,7 +3052,7 @@
           <t>Software / ML engineer</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="18" t="n">
@@ -2985,23 +3061,23 @@
       <c r="F12" s="19" t="n">
         <v>0.05</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="12">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="12">
         <f>G12*F12</f>
         <v/>
       </c>
-      <c r="I12" s="13">
-        <f>MAX(0,(E12+E12*F12)-Assumptions!$C$30)*Assumptions!$C$29*D12</f>
-        <v/>
-      </c>
-      <c r="J12" s="13">
-        <f>(G12+H12)*(Assumptions!$C$31+Assumptions!$C$32)</f>
-        <v/>
-      </c>
-      <c r="K12" s="13">
+      <c r="I12" s="12">
+        <f>MAX(0,(E12+E12*F12)-Assumptions!$C$33)*Assumptions!$C$32*D12</f>
+        <v/>
+      </c>
+      <c r="J12" s="12">
+        <f>(G12+H12)*(Assumptions!$C$34+Assumptions!$C$35)</f>
+        <v/>
+      </c>
+      <c r="K12" s="12">
         <f>G12+H12+I12+J12</f>
         <v/>
       </c>
@@ -3049,7 +3125,7 @@
         </is>
       </c>
       <c r="K15" s="24">
-        <f>D13*Assumptions!$C$33</f>
+        <f>D13*Assumptions!$C$36</f>
         <v/>
       </c>
     </row>
@@ -3060,7 +3136,7 @@
         </is>
       </c>
       <c r="K16" s="24">
-        <f>D13*Assumptions!$C$34</f>
+        <f>D13*Assumptions!$C$37</f>
         <v/>
       </c>
     </row>
@@ -3071,7 +3147,7 @@
         </is>
       </c>
       <c r="K17" s="24">
-        <f>Assumptions!$C$12*Assumptions!$C$36</f>
+        <f>Assumptions!$C$15*Assumptions!$C$39</f>
         <v/>
       </c>
     </row>
@@ -3082,7 +3158,7 @@
         </is>
       </c>
       <c r="K18" s="24">
-        <f>Assumptions!$C$12*Assumptions!$C$37</f>
+        <f>Assumptions!$C$15*Assumptions!$C$40</f>
         <v/>
       </c>
     </row>
@@ -3093,7 +3169,7 @@
         </is>
       </c>
       <c r="K19" s="24">
-        <f>Assumptions!$C$38</f>
+        <f>Assumptions!$C$41</f>
         <v/>
       </c>
     </row>
@@ -3104,6 +3180,733 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Industry salary benchmarks — London, specialist lender, 2025–26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Research ranges from job ads and salary guides (see Sources). 'Used' is the figure in the headcount sheets; founder input overrides the market midpoint where they differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Used</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Bonus % (mid)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Credit analyst / underwriter</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>37500</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Fame Recruitment ad; talent.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Credit analyst / underwriter</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>55000</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>65000</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>Tandem; Fintelligent job ads — founder: analysts normally under £55k</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Credit analyst / underwriter</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>65000</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>85000</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>exec-appointments; Fintelligent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Credit manager</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>65000</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>72500</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>85000</v>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>not in team</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Fintelligent</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Head of credit</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>115000</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>130000</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>115000</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>jobsite; Morgan McKinley (estimate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Case manager</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Junior/mid</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>not in team</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>NRG ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Completions specialist</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>35000</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>42500</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G12" s="18" t="n">
+        <v>42500</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Stellar Select (London uplift estimated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Loan administrator / servicing</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>26000</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>38000</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <v>32000</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Indeed; PayScale</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Portfolio manager</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Mid/senior</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>57500</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>65000</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <v>57500</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Reed; Fintelligent</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>BDM</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>55000</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>65000</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>Fintelligent; Totaljobs (OTE 1.3–1.8x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Senior BDM / originator</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>85000</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>85000</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Fintelligent; jobsite</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Head of sales</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>110000</v>
+      </c>
+      <c r="F17" s="12" t="n">
+        <v>130000</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>110000</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Glassdoor; bridgingloandirectory (estimate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Marketing executive</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Junior/mid</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>36000</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>43000</v>
+      </c>
+      <c r="G18" s="18" t="n">
+        <v>36000</v>
+      </c>
+      <c r="H18" s="17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Marketing manager</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>41000</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>48000</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>57000</v>
+      </c>
+      <c r="G19" s="18" t="n">
+        <v>48000</v>
+      </c>
+      <c r="H19" s="17" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>CEO / MD</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>C-suite</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>150000</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G20" s="18" t="n">
+        <v>200000</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Exec Capital (estimate; owner-MDs often take less + dividends)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>CFO / FD</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>C-suite</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>110000</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>140000</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>170000</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>140000</v>
+      </c>
+      <c r="H21" s="17" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>FD Capital (estimate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>CTO / Head of technology</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>90000</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>115000</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>140000</v>
+      </c>
+      <c r="G22" s="18" t="n">
+        <v>115000</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Glassdoor (estimate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>COO / Operations director</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>120000</v>
+      </c>
+      <c r="G23" s="18" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Exec Capital (estimate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Software engineer / IT</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>65000</v>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G24" s="18" t="n">
+        <v>65000</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Compliance officer</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Mid/senior</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E25" s="12" t="n">
+        <v>67500</v>
+      </c>
+      <c r="F25" s="12" t="n">
+        <v>75000</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>67500</v>
+      </c>
+      <c r="H25" s="17" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Morgan McKinley 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Employer on-costs used: NI 15% above £5,000; pension 5%; other 8% → fully loaded ≈ 1.28× base + bonus. London desk £9,600/yr.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3149,7 +3952,7 @@
         </is>
       </c>
       <c r="C5" s="24">
-        <f>Assumptions!$C$10</f>
+        <f>Assumptions!$C$13</f>
         <v/>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -3176,8 +3979,8 @@
           <t>Arrangement fee charged (gross)</t>
         </is>
       </c>
-      <c r="C8" s="13">
-        <f>C5*Assumptions!$C$16</f>
+      <c r="C8" s="12">
+        <f>C5*Assumptions!$C$19</f>
         <v/>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -3192,8 +3995,8 @@
           <t>Less: introducer / broker share of arrangement fee</t>
         </is>
       </c>
-      <c r="C9" s="13">
-        <f>-C5*(Assumptions!$C$16-Assumptions!$C$17)*Assumptions!$C$22</f>
+      <c r="C9" s="12">
+        <f>-C5*(Assumptions!$C$19-Assumptions!$C$20)*Assumptions!$C$25</f>
         <v/>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -3208,8 +4011,8 @@
           <t>Gross interest income</t>
         </is>
       </c>
-      <c r="C10" s="13">
-        <f>C6*Assumptions!$C$15</f>
+      <c r="C10" s="12">
+        <f>C6*Assumptions!$C$18</f>
         <v/>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -3225,7 +4028,7 @@
         </is>
       </c>
       <c r="C11" s="24">
-        <f>Assumptions!$C$9*(Assumptions!$C$18+Assumptions!$C$19)</f>
+        <f>Assumptions!$C$12*(Assumptions!$C$21+Assumptions!$C$22)</f>
         <v/>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -3240,8 +4043,8 @@
           <t>Exit fee income</t>
         </is>
       </c>
-      <c r="C12" s="13">
-        <f>C5*Assumptions!$C$20</f>
+      <c r="C12" s="12">
+        <f>C5*Assumptions!$C$23</f>
         <v/>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -3256,8 +4059,8 @@
           <t>Other fee income</t>
         </is>
       </c>
-      <c r="C13" s="13">
-        <f>C5*Assumptions!$C$21</f>
+      <c r="C13" s="12">
+        <f>C5*Assumptions!$C$24</f>
         <v/>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -3272,7 +4075,7 @@
           <t>GROSS REVENUE (after broker share)</t>
         </is>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="12">
         <f>SUM(C8:C13)</f>
         <v/>
       </c>
@@ -3284,8 +4087,8 @@
           <t>Less: cost of funds (funding partner buy rate)</t>
         </is>
       </c>
-      <c r="C16" s="13">
-        <f>-C6*Assumptions!$C$25*Assumptions!$C$24</f>
+      <c r="C16" s="12">
+        <f>-C6*Assumptions!$C$28*Assumptions!$C$27</f>
         <v/>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -3300,8 +4103,8 @@
           <t>Less: funder fees</t>
         </is>
       </c>
-      <c r="C17" s="13">
-        <f>-Assumptions!$C$9*Assumptions!$C$26</f>
+      <c r="C17" s="12">
+        <f>-Assumptions!$C$12*Assumptions!$C$29</f>
         <v/>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -3316,8 +4119,8 @@
           <t>Less: expected credit losses</t>
         </is>
       </c>
-      <c r="C18" s="13">
-        <f>-C6*Assumptions!$C$27</f>
+      <c r="C18" s="12">
+        <f>-C6*Assumptions!$C$30</f>
         <v/>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -3332,7 +4135,7 @@
           <t>NET REVENUE (after funding, brokers, losses)</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="12">
         <f>C14+SUM(C16:C18)</f>
         <v/>
       </c>
@@ -3348,7 +4151,7 @@
           <t>Net revenue as % of book</t>
         </is>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="17">
         <f>C19/C6</f>
         <v/>
       </c>
@@ -3360,8 +4163,8 @@
           <t>Net revenue per completed loan</t>
         </is>
       </c>
-      <c r="C22" s="13">
-        <f>C19/Assumptions!$C$9</f>
+      <c r="C22" s="12">
+        <f>C19/Assumptions!$C$12</f>
         <v/>
       </c>
       <c r="D22" s="9" t="inlineStr"/>
@@ -3372,7 +4175,7 @@
           <t>Net interest margin (% of book)</t>
         </is>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="17">
         <f>(C10+C16)/C6</f>
         <v/>
       </c>
@@ -3387,7 +4190,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3467,7 +4270,7 @@
         <f>'Headcount - AI-native'!K13</f>
         <v/>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="12">
         <f>D6-C6</f>
         <v/>
       </c>
@@ -3491,7 +4294,7 @@
         <f>'Headcount - AI-native'!K15</f>
         <v/>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="12">
         <f>D7-C7</f>
         <v/>
       </c>
@@ -3510,7 +4313,7 @@
         <f>'Headcount - AI-native'!K16</f>
         <v/>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="12">
         <f>D8-C8</f>
         <v/>
       </c>
@@ -3529,7 +4332,7 @@
         <f>'Headcount - AI-native'!K18</f>
         <v/>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="12">
         <f>D9-C9</f>
         <v/>
       </c>
@@ -3548,7 +4351,7 @@
         <f>'Headcount - AI-native'!K17</f>
         <v/>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="12">
         <f>D10-C10</f>
         <v/>
       </c>
@@ -3567,7 +4370,7 @@
         <f>'Headcount - AI-native'!K19</f>
         <v/>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="12">
         <f>D11-C11</f>
         <v/>
       </c>
@@ -3610,7 +4413,7 @@
         <f>Revenue!C19</f>
         <v/>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="12">
         <f>D14-C14</f>
         <v/>
       </c>
@@ -3629,7 +4432,7 @@
         <f>D14-D12</f>
         <v/>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="12">
         <f>D15-C15</f>
         <v/>
       </c>
@@ -3648,7 +4451,7 @@
         <f>D15/D14</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="17">
         <f>D16-C16</f>
         <v/>
       </c>
@@ -3660,11 +4463,11 @@
         </is>
       </c>
       <c r="C18" s="30">
-        <f>Assumptions!$C$9</f>
+        <f>Assumptions!$C$12</f>
         <v/>
       </c>
       <c r="D18" s="30">
-        <f>Assumptions!$C$9</f>
+        <f>Assumptions!$C$12</f>
         <v/>
       </c>
     </row>
@@ -3675,14 +4478,14 @@
         </is>
       </c>
       <c r="C19" s="24">
-        <f>C12/Assumptions!$C$9</f>
+        <f>C12/Assumptions!$C$12</f>
         <v/>
       </c>
       <c r="D19" s="24">
-        <f>D12/Assumptions!$C$9</f>
-        <v/>
-      </c>
-      <c r="E19" s="13">
+        <f>D12/Assumptions!$C$12</f>
+        <v/>
+      </c>
+      <c r="E19" s="12">
         <f>D19-C19</f>
         <v/>
       </c>
@@ -3699,11 +4502,11 @@
         </is>
       </c>
       <c r="C20" s="31">
-        <f>C12/Assumptions!$C$10</f>
+        <f>C12/Assumptions!$C$13</f>
         <v/>
       </c>
       <c r="D20" s="31">
-        <f>D12/Assumptions!$C$10</f>
+        <f>D12/Assumptions!$C$13</f>
         <v/>
       </c>
       <c r="E20" s="32">
@@ -3730,7 +4533,7 @@
         <f>Assumptions!$C$6/D5</f>
         <v/>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="12">
         <f>D21-C21</f>
         <v/>
       </c>
@@ -3742,11 +4545,11 @@
         </is>
       </c>
       <c r="C22" s="25">
-        <f>Assumptions!$C$9/C5</f>
+        <f>Assumptions!$C$12/C5</f>
         <v/>
       </c>
       <c r="D22" s="25">
-        <f>Assumptions!$C$9/D5</f>
+        <f>Assumptions!$C$12/D5</f>
         <v/>
       </c>
       <c r="E22" s="26">
@@ -3841,16 +4644,16 @@
           <t>Loans completed per year</t>
         </is>
       </c>
-      <c r="C30" s="12">
-        <f>ROUND(Assumptions!$C$9*C29,0)</f>
-        <v/>
-      </c>
-      <c r="D30" s="12">
-        <f>ROUND(Assumptions!$C$9*D29,0)</f>
-        <v/>
-      </c>
-      <c r="E30" s="12">
-        <f>ROUND(Assumptions!$C$9*E29,0)</f>
+      <c r="C30" s="14">
+        <f>ROUND(Assumptions!$C$12*C29,0)</f>
+        <v/>
+      </c>
+      <c r="D30" s="14">
+        <f>ROUND(Assumptions!$C$12*D29,0)</f>
+        <v/>
+      </c>
+      <c r="E30" s="14">
+        <f>ROUND(Assumptions!$C$12*E29,0)</f>
         <v/>
       </c>
     </row>
@@ -3860,15 +4663,15 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="C31" s="13">
+      <c r="C31" s="12">
         <f>Revenue!$C$19*C29</f>
         <v/>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="12">
         <f>Revenue!$C$19*D29</f>
         <v/>
       </c>
-      <c r="E31" s="13">
+      <c r="E31" s="12">
         <f>Revenue!$C$19*E29</f>
         <v/>
       </c>
@@ -3905,16 +4708,16 @@
           <t>Operating cost</t>
         </is>
       </c>
-      <c r="C35" s="13">
-        <f>SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23)+('Headcount - Traditional'!$K$24-SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23))*C29+C34*(Assumptions!$C$33+Assumptions!$C$34)+Assumptions!$C$12*C29*Assumptions!$C$37</f>
-        <v/>
-      </c>
-      <c r="D35" s="13">
-        <f>SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23)+('Headcount - Traditional'!$K$24-SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23))*D29+D34*(Assumptions!$C$33+Assumptions!$C$34)+Assumptions!$C$12*D29*Assumptions!$C$37</f>
-        <v/>
-      </c>
-      <c r="E35" s="13">
-        <f>SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23)+('Headcount - Traditional'!$K$24-SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23))*E29+E34*(Assumptions!$C$33+Assumptions!$C$34)+Assumptions!$C$12*E29*Assumptions!$C$37</f>
+      <c r="C35" s="12">
+        <f>SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23)+('Headcount - Traditional'!$K$24-SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23))*C29+C34*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$15*C29*Assumptions!$C$40</f>
+        <v/>
+      </c>
+      <c r="D35" s="12">
+        <f>SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23)+('Headcount - Traditional'!$K$24-SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23))*D29+D34*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$15*D29*Assumptions!$C$40</f>
+        <v/>
+      </c>
+      <c r="E35" s="12">
+        <f>SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23)+('Headcount - Traditional'!$K$24-SUMIF('Headcount - Traditional'!B6:B23,"Management",'Headcount - Traditional'!K6:K23))*E29+E34*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$15*E29*Assumptions!$C$40</f>
         <v/>
       </c>
     </row>
@@ -3924,15 +4727,15 @@
           <t>Operating profit</t>
         </is>
       </c>
-      <c r="C36" s="13">
+      <c r="C36" s="12">
         <f>C31-C35</f>
         <v/>
       </c>
-      <c r="D36" s="13">
+      <c r="D36" s="12">
         <f>D31-D35</f>
         <v/>
       </c>
-      <c r="E36" s="13">
+      <c r="E36" s="12">
         <f>E31-E35</f>
         <v/>
       </c>
@@ -3943,15 +4746,15 @@
           <t>Operating margin</t>
         </is>
       </c>
-      <c r="C37" s="16">
+      <c r="C37" s="17">
         <f>C36/C31</f>
         <v/>
       </c>
-      <c r="D37" s="16">
+      <c r="D37" s="17">
         <f>D36/D31</f>
         <v/>
       </c>
-      <c r="E37" s="16">
+      <c r="E37" s="17">
         <f>E36/E31</f>
         <v/>
       </c>
@@ -3962,15 +4765,15 @@
           <t>Cost per completed loan</t>
         </is>
       </c>
-      <c r="C38" s="13">
+      <c r="C38" s="12">
         <f>C35/C30</f>
         <v/>
       </c>
-      <c r="D38" s="13">
+      <c r="D38" s="12">
         <f>D35/D30</f>
         <v/>
       </c>
-      <c r="E38" s="13">
+      <c r="E38" s="12">
         <f>E35/E30</f>
         <v/>
       </c>
@@ -4007,16 +4810,16 @@
           <t>Operating cost</t>
         </is>
       </c>
-      <c r="C42" s="13">
-        <f>(SUM('Headcount - AI-native'!K6:K12)-'Headcount - AI-native'!K8-'Headcount - AI-native'!K11)+ROUNDUP(C28/75000000,0)*('Headcount - AI-native'!K8/'Headcount - AI-native'!D8)+ROUNDUP(C28/150000000,0)*('Headcount - AI-native'!K11/'Headcount - AI-native'!D11)+C41*(Assumptions!$C$33+Assumptions!$C$34)+Assumptions!$C$12*C29*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$38*(1+0.5*(C29-1))</f>
-        <v/>
-      </c>
-      <c r="D42" s="13">
-        <f>(SUM('Headcount - AI-native'!K6:K12)-'Headcount - AI-native'!K8-'Headcount - AI-native'!K11)+ROUNDUP(D28/75000000,0)*('Headcount - AI-native'!K8/'Headcount - AI-native'!D8)+ROUNDUP(D28/150000000,0)*('Headcount - AI-native'!K11/'Headcount - AI-native'!D11)+D41*(Assumptions!$C$33+Assumptions!$C$34)+Assumptions!$C$12*D29*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$38*(1+0.5*(D29-1))</f>
-        <v/>
-      </c>
-      <c r="E42" s="13">
-        <f>(SUM('Headcount - AI-native'!K6:K12)-'Headcount - AI-native'!K8-'Headcount - AI-native'!K11)+ROUNDUP(E28/75000000,0)*('Headcount - AI-native'!K8/'Headcount - AI-native'!D8)+ROUNDUP(E28/150000000,0)*('Headcount - AI-native'!K11/'Headcount - AI-native'!D11)+E41*(Assumptions!$C$33+Assumptions!$C$34)+Assumptions!$C$12*E29*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$38*(1+0.5*(E29-1))</f>
+      <c r="C42" s="12">
+        <f>(SUM('Headcount - AI-native'!K6:K12)-'Headcount - AI-native'!K8-'Headcount - AI-native'!K11)+ROUNDUP(C28/75000000,0)*('Headcount - AI-native'!K8/'Headcount - AI-native'!D8)+ROUNDUP(C28/150000000,0)*('Headcount - AI-native'!K11/'Headcount - AI-native'!D11)+C41*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$15*C29*(Assumptions!$C$39+Assumptions!$C$40)+Assumptions!$C$41*(1+0.5*(C29-1))</f>
+        <v/>
+      </c>
+      <c r="D42" s="12">
+        <f>(SUM('Headcount - AI-native'!K6:K12)-'Headcount - AI-native'!K8-'Headcount - AI-native'!K11)+ROUNDUP(D28/75000000,0)*('Headcount - AI-native'!K8/'Headcount - AI-native'!D8)+ROUNDUP(D28/150000000,0)*('Headcount - AI-native'!K11/'Headcount - AI-native'!D11)+D41*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$15*D29*(Assumptions!$C$39+Assumptions!$C$40)+Assumptions!$C$41*(1+0.5*(D29-1))</f>
+        <v/>
+      </c>
+      <c r="E42" s="12">
+        <f>(SUM('Headcount - AI-native'!K6:K12)-'Headcount - AI-native'!K8-'Headcount - AI-native'!K11)+ROUNDUP(E28/75000000,0)*('Headcount - AI-native'!K8/'Headcount - AI-native'!D8)+ROUNDUP(E28/150000000,0)*('Headcount - AI-native'!K11/'Headcount - AI-native'!D11)+E41*(Assumptions!$C$36+Assumptions!$C$37)+Assumptions!$C$15*E29*(Assumptions!$C$39+Assumptions!$C$40)+Assumptions!$C$41*(1+0.5*(E29-1))</f>
         <v/>
       </c>
       <c r="F42" s="9" t="inlineStr">
@@ -4031,15 +4834,15 @@
           <t>Operating profit</t>
         </is>
       </c>
-      <c r="C43" s="13">
+      <c r="C43" s="12">
         <f>C31-C42</f>
         <v/>
       </c>
-      <c r="D43" s="13">
+      <c r="D43" s="12">
         <f>D31-D42</f>
         <v/>
       </c>
-      <c r="E43" s="13">
+      <c r="E43" s="12">
         <f>E31-E42</f>
         <v/>
       </c>
@@ -4050,15 +4853,15 @@
           <t>Operating margin</t>
         </is>
       </c>
-      <c r="C44" s="16">
+      <c r="C44" s="17">
         <f>C43/C31</f>
         <v/>
       </c>
-      <c r="D44" s="16">
+      <c r="D44" s="17">
         <f>D43/D31</f>
         <v/>
       </c>
-      <c r="E44" s="16">
+      <c r="E44" s="17">
         <f>E43/E31</f>
         <v/>
       </c>
@@ -4069,15 +4872,15 @@
           <t>Cost per completed loan</t>
         </is>
       </c>
-      <c r="C45" s="13">
+      <c r="C45" s="12">
         <f>C42/C30</f>
         <v/>
       </c>
-      <c r="D45" s="13">
+      <c r="D45" s="12">
         <f>D42/D30</f>
         <v/>
       </c>
-      <c r="E45" s="13">
+      <c r="E45" s="12">
         <f>E42/E30</f>
         <v/>
       </c>
@@ -4125,7 +4928,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4177,11 +4980,11 @@
         </is>
       </c>
       <c r="C5" s="24">
-        <f>SUM('Headcount - Traditional'!K7:K8)/SUM('Headcount - Traditional'!D7:D8)/Assumptions!$C$41</f>
+        <f>SUM('Headcount - Traditional'!K7:K8)/SUM('Headcount - Traditional'!D7:D8)/Assumptions!$C$44</f>
         <v/>
       </c>
       <c r="D5" s="24">
-        <f>SUM('Headcount - Traditional'!K7:K8)/SUM('Headcount - Traditional'!D7:D8)/Assumptions!$C$41</f>
+        <f>SUM('Headcount - Traditional'!K7:K8)/SUM('Headcount - Traditional'!D7:D8)/Assumptions!$C$44</f>
         <v/>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -4197,11 +5000,11 @@
         </is>
       </c>
       <c r="C6" s="25">
-        <f>Assumptions!$C$40</f>
+        <f>Assumptions!$C$43</f>
         <v/>
       </c>
       <c r="D6" s="25">
-        <f>Assumptions!$C$39</f>
+        <f>Assumptions!$C$42</f>
         <v/>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -4237,7 +5040,7 @@
         <v/>
       </c>
       <c r="D8" s="24">
-        <f>Assumptions!$C$36</f>
+        <f>Assumptions!$C$39</f>
         <v/>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -4253,11 +5056,11 @@
         </is>
       </c>
       <c r="C9" s="24">
-        <f>Assumptions!$C$37</f>
+        <f>Assumptions!$C$40</f>
         <v/>
       </c>
       <c r="D9" s="24">
-        <f>Assumptions!$C$37</f>
+        <f>Assumptions!$C$40</f>
         <v/>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -4289,11 +5092,11 @@
         </is>
       </c>
       <c r="C12" s="30">
-        <f>Assumptions!$C$41/C6</f>
+        <f>Assumptions!$C$44/C6</f>
         <v/>
       </c>
       <c r="D12" s="30">
-        <f>Assumptions!$C$41/D6</f>
+        <f>Assumptions!$C$44/D6</f>
         <v/>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -4308,10 +5111,10 @@
           <t>Elapsed time to first credit view</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <v>0.25</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -4337,7 +5140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>